<commit_message>
feat(decision-helper-service): F-011..F-016 — Phase B signal engine complete
- F-011: DB schema already in domain.py; marked Done in roadmap
- F-012: regime/classifier.py — fetches analysis-service regime, maps
         TREND→TREND_UP/TREND_DOWN by MA slope sign
- F-013: signal/trend/ma_cross.py — fast/slow SMA crossover detector
- F-014: signal/trend/n_day_breakout.py — N-day high/low breakout
- F-015: signal/range/sr_bounce_breakout.py — SR bounce + breakout signals
- F-016: confirmation/layer.py — penetration %, time-delay K bars,
         oscillator-as-alert (RSI) rule (Schwager Ch 6/7/14)
- services/market/client.py — async HTTP façade over analysis-service,
  stock-data-service, ai-insights-service
- POST /helper/signal-analysis endpoint wired in routes.py
- road_map_version_11.xlsx: F-011..F-016 → Done, Phase B → Done

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/road_map_version_11.xlsx
+++ b/stockpredict/road_map_version_11.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>